<commit_message>
rerun and update line ends
</commit_message>
<xml_diff>
--- a/output_data/charts/0500000US39041.xlsx
+++ b/output_data/charts/0500000US39041.xlsx
@@ -161,47 +161,32 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$14</c:f>
+              <c:f>Sheet1!$A$2:$A$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>2012</c:v>
+                  <c:v>2017</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2013</c:v>
+                  <c:v>2018</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2014</c:v>
+                  <c:v>2019</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2015</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2016</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2017</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2018</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2019</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>2020</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>2021</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>2022</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="12">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -209,47 +194,32 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$14</c:f>
+              <c:f>Sheet1!$B$2:$B$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>4.655580178401832</c:v>
+                  <c:v>4.794241264663446</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.621017400469683</c:v>
+                  <c:v>5.074002373071879</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.610526689255114</c:v>
+                  <c:v>5.050627166812981</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.672463568875447</c:v>
+                  <c:v>5.501011766469309</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.643911500315123</c:v>
+                  <c:v>5.707206392071159</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.798946113794617</c:v>
+                  <c:v>6.004460456338995</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5.074002373071879</c:v>
+                  <c:v>6.299263470732653</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.038537652327882</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>5.501011766469309</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>5.707206392071159</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>6.004460456338995</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>6.299263470732653</c:v>
-                </c:pt>
-                <c:pt idx="12">
                   <c:v>6.028599676867057</c:v>
                 </c:pt>
               </c:numCache>
@@ -676,7 +646,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" style="1" customWidth="1"/>
@@ -692,105 +662,65 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>2012</v>
+        <v>2017</v>
       </c>
       <c r="B2" s="1">
-        <v>4.655580178401832</v>
+        <v>4.794241264663446</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>2013</v>
+        <v>2018</v>
       </c>
       <c r="B3" s="1">
-        <v>4.621017400469683</v>
+        <v>5.074002373071879</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>2014</v>
+        <v>2019</v>
       </c>
       <c r="B4" s="1">
-        <v>4.610526689255114</v>
+        <v>5.050627166812981</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="B5" s="1">
-        <v>4.672463568875447</v>
+        <v>5.501011766469309</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>2016</v>
+        <v>2021</v>
       </c>
       <c r="B6" s="1">
-        <v>4.643911500315123</v>
+        <v>5.707206392071159</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>2017</v>
+        <v>2022</v>
       </c>
       <c r="B7" s="1">
-        <v>4.798946113794617</v>
+        <v>6.004460456338995</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="B8" s="1">
-        <v>5.074002373071879</v>
+        <v>6.299263470732653</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>2019</v>
+        <v>2024</v>
       </c>
       <c r="B9" s="1">
-        <v>5.038537652327882</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="2">
-        <v>2020</v>
-      </c>
-      <c r="B10" s="1">
-        <v>5.501011766469309</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="2">
-        <v>2021</v>
-      </c>
-      <c r="B11" s="1">
-        <v>5.707206392071159</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="2">
-        <v>2022</v>
-      </c>
-      <c r="B12" s="1">
-        <v>6.004460456338995</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="2">
-        <v>2023</v>
-      </c>
-      <c r="B13" s="1">
-        <v>6.299263470732653</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14" s="2">
-        <v>2024</v>
-      </c>
-      <c r="B14" s="1">
         <v>6.028599676867057</v>
       </c>
     </row>

</xml_diff>

<commit_message>
rerun pipeline with all years
</commit_message>
<xml_diff>
--- a/output_data/charts/0500000US39041.xlsx
+++ b/output_data/charts/0500000US39041.xlsx
@@ -161,32 +161,47 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$9</c:f>
+              <c:f>Sheet1!$A$2:$A$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
+                  <c:v>2012</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2013</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2014</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2015</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2016</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>2017</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="6">
                   <c:v>2018</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="7">
                   <c:v>2019</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="8">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="9">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="10">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="11">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="12">
                   <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
@@ -194,32 +209,47 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$9</c:f>
+              <c:f>Sheet1!$B$2:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
+                  <c:v>4.748691781969869</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.732890770909226</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.612300651043976</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.663089428100083</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.643911500315123</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>4.794241264663446</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="6">
                   <c:v>5.074002373071879</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="7">
                   <c:v>5.050627166812981</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="8">
                   <c:v>5.501011766469309</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="9">
                   <c:v>5.707206392071159</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="10">
                   <c:v>6.004460456338995</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="11">
                   <c:v>6.299263470732653</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="12">
                   <c:v>6.028599676867057</c:v>
                 </c:pt>
               </c:numCache>
@@ -646,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" style="1" customWidth="1"/>
@@ -662,65 +692,105 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>2017</v>
+        <v>2012</v>
       </c>
       <c r="B2" s="1">
-        <v>4.794241264663446</v>
+        <v>4.748691781969869</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>2018</v>
+        <v>2013</v>
       </c>
       <c r="B3" s="1">
-        <v>5.074002373071879</v>
+        <v>4.732890770909226</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="B4" s="1">
-        <v>5.050627166812981</v>
+        <v>4.612300651043976</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="B5" s="1">
-        <v>5.501011766469309</v>
+        <v>4.663089428100083</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>2021</v>
+        <v>2016</v>
       </c>
       <c r="B6" s="1">
-        <v>5.707206392071159</v>
+        <v>4.643911500315123</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="B7" s="1">
-        <v>6.004460456338995</v>
+        <v>4.794241264663446</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="B8" s="1">
-        <v>6.299263470732653</v>
+        <v>5.074002373071879</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
+        <v>2019</v>
+      </c>
+      <c r="B9" s="1">
+        <v>5.050627166812981</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="2">
+        <v>2020</v>
+      </c>
+      <c r="B10" s="1">
+        <v>5.501011766469309</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="2">
+        <v>2021</v>
+      </c>
+      <c r="B11" s="1">
+        <v>5.707206392071159</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="2">
+        <v>2022</v>
+      </c>
+      <c r="B12" s="1">
+        <v>6.004460456338995</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="2">
+        <v>2023</v>
+      </c>
+      <c r="B13" s="1">
+        <v>6.299263470732653</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="2">
         <v>2024</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B14" s="1">
         <v>6.028599676867057</v>
       </c>
     </row>

</xml_diff>